<commit_message>
Add LC-MS phenolics outcomes to DOE
</commit_message>
<xml_diff>
--- a/dashboard/doe_assets/initial_doe_workbook.xlsx
+++ b/dashboard/doe_assets/initial_doe_workbook.xlsx
@@ -13,8 +13,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20-run matrix'!$A$1:$O$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'data dictionary'!$A$1:$E$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'sampling matrix'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'data dictionary'!$A$1:$E$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'sampling matrix'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1649,11 +1649,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
@@ -2801,17 +2801,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>sensory_offodor_score</t>
+          <t>total_phenolics</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Calibrated off-odor score</t>
+          <t>Total phenolic content</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>prespecified scale</t>
+          <t>validated assay unit</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2823,135 +2823,135 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>QC and feasibility</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>instrument_batch</t>
+          <t>phenolic_profile_LCMS</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Analytical batch identifier</t>
+          <t>Individual phenolic acids and flavonoids by LC-MS</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>validated concentration basis</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>record actual</t>
+          <t>selected subset</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>QC and feasibility</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>qc_flag</t>
+          <t>chlorophyll_related_profile_LCMS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PASS, WARN, or FAIL</t>
+          <t>Chlorophyll-related compounds and degradation products by LC-MS</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>validated concentration basis</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>selected subset</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>QC and feasibility</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>lod_state</t>
+          <t>sensory_offodor_score</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Measured, below LOQ, or below LOD</t>
+          <t>Calibrated off-odor score</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>prespecified scale</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Measured</t>
+          <t>selected subset</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>QC and feasibility</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>energy_kWh</t>
+          <t>sensory_bitterness_score</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Measured process energy</t>
+          <t>Calibrated bitterness score</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>kWh</t>
+          <t>prespecified scale</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>record actual</t>
+          <t>selected subset</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>QC and feasibility</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>water_L</t>
+          <t>sensory_astringency_score</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Water used</t>
+          <t>Calibrated astringency score</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>prespecified scale</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>record actual</t>
+          <t>selected subset</t>
         </is>
       </c>
     </row>
@@ -2963,17 +2963,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>chemical_cost_ILS</t>
+          <t>instrument_batch</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Treatment chemical cost</t>
+          <t>Analytical batch identifier</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ILS</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2990,27 +2990,162 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>qc_flag</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>PASS, WARN, or FAIL</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>QC and feasibility</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>lod_state</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Measured, below LOQ, or below LOD</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Measured</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>QC and feasibility</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>energy_kWh</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Measured process energy</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>record actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>QC and feasibility</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>water_L</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Water used</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>record actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>QC and feasibility</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>chemical_cost_ILS</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Treatment chemical cost</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>record actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>QC and feasibility</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>labor_time_min</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Hands-on labor</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>record actual</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E50"/>
+  <autoFilter ref="A1:E55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3021,11 +3156,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -3180,24 +3315,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>L*, a*, b*</t>
+          <t>LC-MS phenolic profile</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required baseline</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
+          <t>Selected subset</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Required</t>
@@ -3207,12 +3338,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chlorophyll</t>
+          <t>LC-MS chlorophyll-related profile</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Required baseline</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3220,11 +3351,7 @@
           <t>Selected subset</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Selected subset</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Required</t>
@@ -3234,24 +3361,93 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>L*, a*, b*</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Chlorophyll</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Selected subset</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Selected subset</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Sensory off-odor</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
         <is>
           <t>Selected subset</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Selected subset</t>
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sensory bitterness/astringency</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Selected subset</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align DOE with thermal volatiles plan
</commit_message>
<xml_diff>
--- a/dashboard/doe_assets/initial_doe_workbook.xlsx
+++ b/dashboard/doe_assets/initial_doe_workbook.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20-run matrix'!$A$1:$O$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'data dictionary'!$A$1:$E$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'data dictionary'!$A$1:$E$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'sampling matrix'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1649,14 +1649,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2639,22 +2639,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>protein_recovery_pct</t>
+          <t>thermal_volatiles_T2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Recovered protein relative to starting protein</t>
+          <t>Thermally generated volatiles, including annotated pyrazines, in dried product</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>validated concentration basis</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>critical constraint</t>
+          <t>secondary/exploratory; required measurement</t>
         </is>
       </c>
     </row>
@@ -2666,17 +2666,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>protein_content_pct_DM</t>
+          <t>protein_recovery_pct</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Final product protein content</t>
+          <t>Recovered protein relative to starting protein</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>% DM</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2693,22 +2693,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>color_L</t>
+          <t>protein_content_pct_DM</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CIE lightness</t>
+          <t>Final product protein content</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>CIE L*</t>
+          <t>% DM</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>required</t>
+          <t>critical constraint</t>
         </is>
       </c>
     </row>
@@ -2720,17 +2720,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>color_a</t>
+          <t>color_L</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CIE red-green coordinate</t>
+          <t>CIE lightness</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CIE a*</t>
+          <t>CIE L*</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2747,17 +2747,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>color_b</t>
+          <t>color_a</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CIE yellow-blue coordinate</t>
+          <t>CIE red-green coordinate</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CIE b*</t>
+          <t>CIE a*</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2774,22 +2774,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>chlorophyll_total</t>
+          <t>color_b</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Total chlorophyll</t>
+          <t>CIE yellow-blue coordinate</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>validated assay unit</t>
+          <t>CIE b*</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>selected subset</t>
+          <t>required</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2801,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>total_phenolics</t>
+          <t>chlorophyll_total</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Total phenolic content</t>
+          <t>Total chlorophyll</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2828,17 +2828,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>phenolic_profile_LCMS</t>
+          <t>total_phenolics</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Individual phenolic acids and flavonoids by LC-MS</t>
+          <t>Total phenolic content</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>validated concentration basis</t>
+          <t>validated assay unit</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2855,12 +2855,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>chlorophyll_related_profile_LCMS</t>
+          <t>phenolic_profile_LCMS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Chlorophyll-related compounds and degradation products by LC-MS</t>
+          <t>Individual phenolic acids and flavonoids by LC-MS</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2882,17 +2882,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>sensory_offodor_score</t>
+          <t>chlorophyll_related_profile_LCMS</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Calibrated off-odor score</t>
+          <t>Chlorophyll-related compounds and degradation products by LC-MS</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>prespecified scale</t>
+          <t>validated concentration basis</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2909,12 +2909,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>sensory_bitterness_score</t>
+          <t>sensory_offodor_score</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Calibrated bitterness score</t>
+          <t>Calibrated off-odor score</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2936,12 +2936,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>sensory_astringency_score</t>
+          <t>sensory_bitterness_score</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Calibrated astringency score</t>
+          <t>Calibrated bitterness score</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2958,27 +2958,27 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>QC and feasibility</t>
+          <t>Outcomes</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>instrument_batch</t>
+          <t>sensory_astringency_score</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Analytical batch identifier</t>
+          <t>Calibrated astringency score</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>prespecified scale</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>record actual</t>
+          <t>selected subset</t>
         </is>
       </c>
     </row>
@@ -2990,22 +2990,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>qc_flag</t>
+          <t>instrument_batch</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PASS, WARN, or FAIL</t>
+          <t>Analytical batch identifier</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>record actual</t>
         </is>
       </c>
     </row>
@@ -3017,12 +3017,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>lod_state</t>
+          <t>qc_flag</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Measured, below LOQ, or below LOD</t>
+          <t>PASS, WARN, or FAIL</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Measured</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -3044,22 +3044,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>energy_kWh</t>
+          <t>lod_state</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Measured process energy</t>
+          <t>Measured, below LOQ, or below LOD</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>kWh</t>
+          <t>category</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>record actual</t>
+          <t>Measured</t>
         </is>
       </c>
     </row>
@@ -3071,17 +3071,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>water_L</t>
+          <t>energy_kWh</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Water used</t>
+          <t>Measured process energy</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>kWh</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3098,17 +3098,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>chemical_cost_ILS</t>
+          <t>water_L</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Treatment chemical cost</t>
+          <t>Water used</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ILS</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3125,27 +3125,54 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>chemical_cost_ILS</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Treatment chemical cost</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ILS</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>record actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>QC and feasibility</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>labor_time_min</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Hands-on labor</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>record actual</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E55"/>
+  <autoFilter ref="A1:E56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3292,7 +3319,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GC-MS C6 compounds</t>
+          <t>GC-MS C6 and other volatiles</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -3308,7 +3335,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Recommended</t>
+          <t>Required</t>
         </is>
       </c>
     </row>

</xml_diff>